<commit_message>
docs: add thesis proposal, EXP-003, and project backup
Include expanded 开题报告 output with verified bibliography, EXP-003 experiment record, Model 3.0 and SPAN data updates, and reference PDFs. Remove large local video archive from tracking.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/01_Data/Simio_Import_Data-SPAN.xlsx
+++ b/01_Data/Simio_Import_Data-SPAN.xlsx
@@ -2346,39 +2346,39 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2">
-        <v>39551295</v>
+        <v>39556108</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C2">
-        <v>29092</v>
+        <v>24321</v>
       </c>
       <c r="D2" s="2">
         <v>46023</v>
       </c>
       <c r="E2">
-        <v>120</v>
+        <v>24</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3">
-        <v>39556108</v>
+        <v>39557307</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
       </c>
       <c r="C3">
-        <v>24321</v>
+        <v>45315</v>
       </c>
       <c r="D3" s="2">
         <v>46023</v>
@@ -2398,13 +2398,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4">
-        <v>39557307</v>
+        <v>39557829</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
       <c r="C4">
-        <v>45315</v>
+        <v>118</v>
       </c>
       <c r="D4" s="2">
         <v>46023</v>
@@ -2424,45 +2424,45 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5">
-        <v>39557829</v>
+        <v>39551295</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C5">
-        <v>118</v>
+        <v>29092</v>
       </c>
       <c r="D5" s="2">
         <v>46023</v>
       </c>
       <c r="E5">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H5">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
-        <v>39595805</v>
+        <v>39761062</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>12264</v>
+        <v>7761</v>
       </c>
       <c r="D6" s="2">
         <v>46023</v>
       </c>
       <c r="E6">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -2476,19 +2476,19 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
-        <v>39761060</v>
+        <v>39560050</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C7">
-        <v>6249</v>
+        <v>10232</v>
       </c>
       <c r="D7" s="2">
         <v>46023</v>
       </c>
       <c r="E7">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -2502,13 +2502,13 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8">
-        <v>39761062</v>
+        <v>39762318</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>7761</v>
+        <v>110110</v>
       </c>
       <c r="D8" s="2">
         <v>46023</v>
@@ -2520,21 +2520,21 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9">
-        <v>39560050</v>
+        <v>39567604</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9">
-        <v>10232</v>
+        <v>309997</v>
       </c>
       <c r="D9" s="2">
         <v>46023</v>
@@ -2546,105 +2546,105 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10">
-        <v>39558090</v>
+        <v>39595266</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C10">
-        <v>2400</v>
+        <v>30030</v>
       </c>
       <c r="D10" s="2">
         <v>46023</v>
       </c>
       <c r="E10">
-        <v>312</v>
+        <v>120</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11">
-        <v>39549836</v>
+        <v>39565560</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11">
-        <v>44471</v>
+        <v>60519</v>
       </c>
       <c r="D11" s="2">
         <v>46023</v>
       </c>
       <c r="E11">
-        <v>192</v>
+        <v>120</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12">
-        <v>39561718</v>
+        <v>39561229</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12">
-        <v>26257</v>
+        <v>245001</v>
       </c>
       <c r="D12" s="2">
         <v>46023</v>
       </c>
       <c r="E12">
-        <v>192</v>
+        <v>120</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13">
-        <v>39560730</v>
+        <v>39560930</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C13">
-        <v>679</v>
+        <v>40821</v>
       </c>
       <c r="D13" s="2">
         <v>46023</v>
       </c>
       <c r="E13">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -2658,247 +2658,247 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14">
-        <v>39563480</v>
+        <v>39567605</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C14">
-        <v>373</v>
+        <v>245002</v>
       </c>
       <c r="D14" s="2">
         <v>46023</v>
       </c>
       <c r="E14">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15">
-        <v>39563836</v>
+        <v>39568872</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C15">
-        <v>11382</v>
+        <v>20957</v>
       </c>
       <c r="D15" s="2">
         <v>46023</v>
       </c>
       <c r="E15">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H15">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16">
-        <v>39569477</v>
+        <v>39595805</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C16">
-        <v>50000</v>
+        <v>12264</v>
       </c>
       <c r="D16" s="2">
         <v>46023</v>
       </c>
       <c r="E16">
-        <v>360</v>
+        <v>168</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17">
-        <v>39762318</v>
+        <v>39761060</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C17">
-        <v>110110</v>
+        <v>6249</v>
       </c>
       <c r="D17" s="2">
         <v>46023</v>
       </c>
       <c r="E17">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18">
-        <v>39762322</v>
+        <v>39560730</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C18">
-        <v>30000</v>
+        <v>679</v>
       </c>
       <c r="D18" s="2">
         <v>46023</v>
       </c>
       <c r="E18">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19">
-        <v>39597248</v>
+        <v>39563480</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C19">
-        <v>269556</v>
+        <v>373</v>
       </c>
       <c r="D19" s="2">
         <v>46023</v>
       </c>
       <c r="E19">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20">
-        <v>39564506</v>
+        <v>39563836</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="C20">
-        <v>45000</v>
+        <v>11382</v>
       </c>
       <c r="D20" s="2">
         <v>46023</v>
       </c>
       <c r="E20">
-        <v>360</v>
+        <v>168</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H20">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21">
-        <v>39567604</v>
+        <v>39762319</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C21">
-        <v>309997</v>
+        <v>100010</v>
       </c>
       <c r="D21" s="2">
         <v>46023</v>
       </c>
       <c r="E21">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22">
-        <v>39595266</v>
+        <v>39562366</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C22">
-        <v>30030</v>
+        <v>1484</v>
       </c>
       <c r="D22" s="2">
         <v>46023</v>
       </c>
       <c r="E22">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23">
-        <v>39762319</v>
+        <v>39563481</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C23">
-        <v>100010</v>
+        <v>112</v>
       </c>
       <c r="D23" s="2">
         <v>46023</v>
@@ -2910,307 +2910,307 @@
         <v>1</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H23">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24">
-        <v>39559229</v>
+        <v>39563837</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C24">
-        <v>1454</v>
+        <v>11377</v>
       </c>
       <c r="D24" s="2">
         <v>46023</v>
       </c>
       <c r="E24">
-        <v>240</v>
+        <v>168</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
       <c r="G24">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H24">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25">
-        <v>39562961</v>
+        <v>39565028</v>
       </c>
       <c r="B25" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C25">
-        <v>9401</v>
+        <v>452</v>
       </c>
       <c r="D25" s="2">
         <v>46023</v>
       </c>
       <c r="E25">
-        <v>384</v>
+        <v>168</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H25">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26">
-        <v>39563896</v>
+        <v>39562367</v>
       </c>
       <c r="B26" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C26">
-        <v>193</v>
+        <v>10234</v>
       </c>
       <c r="D26" s="2">
         <v>46023</v>
       </c>
       <c r="E26">
-        <v>384</v>
+        <v>168</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H26">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27">
-        <v>39565146</v>
+        <v>39564593</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C27">
-        <v>10060</v>
+        <v>8820</v>
       </c>
       <c r="D27" s="2">
         <v>46023</v>
       </c>
       <c r="E27">
-        <v>240</v>
+        <v>168</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H27">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28">
-        <v>39560584</v>
+        <v>39549836</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C28">
-        <v>1050</v>
+        <v>44471</v>
       </c>
       <c r="D28" s="2">
         <v>46023</v>
       </c>
       <c r="E28">
-        <v>312</v>
+        <v>192</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H28">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29">
-        <v>39562366</v>
+        <v>39561718</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C29">
-        <v>1484</v>
+        <v>26257</v>
       </c>
       <c r="D29" s="2">
         <v>46023</v>
       </c>
       <c r="E29">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="G29">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30">
-        <v>39563481</v>
+        <v>39762322</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C30">
-        <v>112</v>
+        <v>30000</v>
       </c>
       <c r="D30" s="2">
         <v>46023</v>
       </c>
       <c r="E30">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31">
-        <v>39563837</v>
+        <v>39597248</v>
       </c>
       <c r="B31" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C31">
-        <v>11377</v>
+        <v>269556</v>
       </c>
       <c r="D31" s="2">
         <v>46023</v>
       </c>
       <c r="E31">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32">
-        <v>39565028</v>
+        <v>39559229</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32">
-        <v>452</v>
+        <v>1454</v>
       </c>
       <c r="D32" s="2">
         <v>46023</v>
       </c>
       <c r="E32">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="F32">
         <v>1</v>
       </c>
       <c r="G32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H32">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33">
-        <v>39565560</v>
+        <v>39565146</v>
       </c>
       <c r="B33" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C33">
-        <v>60519</v>
+        <v>10060</v>
       </c>
       <c r="D33" s="2">
         <v>46023</v>
       </c>
       <c r="E33">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
       <c r="G33">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H33">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34">
-        <v>39561229</v>
+        <v>39558090</v>
       </c>
       <c r="B34" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C34">
-        <v>245001</v>
+        <v>2400</v>
       </c>
       <c r="D34" s="2">
         <v>46023</v>
       </c>
       <c r="E34">
-        <v>120</v>
+        <v>312</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H34">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35">
-        <v>39568457</v>
+        <v>39560584</v>
       </c>
       <c r="B35" t="s">
         <v>17</v>
       </c>
       <c r="C35">
-        <v>253</v>
+        <v>1050</v>
       </c>
       <c r="D35" s="2">
         <v>46023</v>
@@ -3230,190 +3230,190 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36">
-        <v>39560930</v>
+        <v>39568457</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C36">
-        <v>40821</v>
+        <v>253</v>
       </c>
       <c r="D36" s="2">
         <v>46023</v>
       </c>
       <c r="E36">
-        <v>120</v>
+        <v>312</v>
       </c>
       <c r="F36">
         <v>1</v>
       </c>
       <c r="G36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H36">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37">
-        <v>39562367</v>
+        <v>39565147</v>
       </c>
       <c r="B37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C37">
-        <v>10234</v>
+        <v>9259</v>
       </c>
       <c r="D37" s="2">
         <v>46023</v>
       </c>
       <c r="E37">
-        <v>168</v>
+        <v>312</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H37">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38">
-        <v>39564593</v>
+        <v>39568458</v>
       </c>
       <c r="B38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C38">
-        <v>8820</v>
+        <v>4340</v>
       </c>
       <c r="D38" s="2">
         <v>46023</v>
       </c>
       <c r="E38">
-        <v>168</v>
+        <v>312</v>
       </c>
       <c r="F38">
         <v>1</v>
       </c>
       <c r="G38">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H38">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39">
-        <v>39565147</v>
+        <v>39569477</v>
       </c>
       <c r="B39" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C39">
-        <v>9259</v>
+        <v>50000</v>
       </c>
       <c r="D39" s="2">
         <v>46023</v>
       </c>
       <c r="E39">
-        <v>312</v>
+        <v>360</v>
       </c>
       <c r="F39">
         <v>1</v>
       </c>
       <c r="G39">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H39">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40">
-        <v>39567605</v>
+        <v>39564506</v>
       </c>
       <c r="B40" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C40">
-        <v>245002</v>
+        <v>45000</v>
       </c>
       <c r="D40" s="2">
         <v>46023</v>
       </c>
       <c r="E40">
-        <v>120</v>
+        <v>360</v>
       </c>
       <c r="F40">
         <v>1</v>
       </c>
       <c r="G40">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41">
-        <v>39568458</v>
+        <v>39562961</v>
       </c>
       <c r="B41" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C41">
-        <v>4340</v>
+        <v>9401</v>
       </c>
       <c r="D41" s="2">
         <v>46023</v>
       </c>
       <c r="E41">
-        <v>312</v>
+        <v>384</v>
       </c>
       <c r="F41">
         <v>1</v>
       </c>
       <c r="G41">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H41">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42">
-        <v>39568872</v>
+        <v>39563896</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C42">
-        <v>20957</v>
+        <v>193</v>
       </c>
       <c r="D42" s="2">
         <v>46023</v>
       </c>
       <c r="E42">
-        <v>144</v>
+        <v>384</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
       <c r="G42">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H42">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H42" etc:filterBottomFollowUsedRange="0">
-    <sortState ref="A1:H42">
-      <sortCondition ref="D1"/>
+    <sortState ref="A2:H42">
+      <sortCondition ref="E1"/>
     </sortState>
     <extLst/>
   </autoFilter>

</xml_diff>